<commit_message>
Bachilleres 1906-07: SEXO en mayúsculas
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Lv8s8TMMsy8TMLZ2ms8p3t
</commit_message>
<xml_diff>
--- a/entregas/Bachilleres_1906-07.xlsx
+++ b/entregas/Bachilleres_1906-07.xlsx
@@ -686,7 +686,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -765,7 +765,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -844,7 +844,7 @@
       <c r="X4" s="2" t="n"/>
       <c r="Y4" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -923,7 +923,7 @@
       <c r="X5" s="2" t="n"/>
       <c r="Y5" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -1002,7 +1002,7 @@
       <c r="X6" s="2" t="n"/>
       <c r="Y6" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1081,7 @@
       <c r="X7" s="2" t="n"/>
       <c r="Y7" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -1160,7 +1160,7 @@
       <c r="X8" s="2" t="n"/>
       <c r="Y8" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -1239,7 +1239,7 @@
       <c r="X9" s="2" t="n"/>
       <c r="Y9" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -1318,7 +1318,7 @@
       <c r="X10" s="2" t="n"/>
       <c r="Y10" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -1397,7 +1397,7 @@
       <c r="X11" s="2" t="n"/>
       <c r="Y11" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -1476,7 +1476,7 @@
       <c r="X12" s="2" t="n"/>
       <c r="Y12" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -1555,7 +1555,7 @@
       <c r="X13" s="2" t="n"/>
       <c r="Y13" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -1634,7 +1634,7 @@
       <c r="X14" s="2" t="n"/>
       <c r="Y14" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -1713,7 +1713,7 @@
       <c r="X15" s="2" t="n"/>
       <c r="Y15" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -1792,7 +1792,7 @@
       <c r="X16" s="2" t="n"/>
       <c r="Y16" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -1871,7 +1871,7 @@
       <c r="X17" s="2" t="n"/>
       <c r="Y17" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -1950,7 +1950,7 @@
       <c r="X18" s="2" t="n"/>
       <c r="Y18" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -2029,7 +2029,7 @@
       <c r="X19" s="2" t="n"/>
       <c r="Y19" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
       <c r="X20" s="2" t="n"/>
       <c r="Y20" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -2187,7 +2187,7 @@
       <c r="X21" s="2" t="n"/>
       <c r="Y21" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -2266,7 +2266,7 @@
       <c r="X22" s="2" t="n"/>
       <c r="Y22" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -2345,7 +2345,7 @@
       <c r="X23" s="2" t="n"/>
       <c r="Y23" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -2424,7 +2424,7 @@
       <c r="X24" s="2" t="n"/>
       <c r="Y24" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -2503,7 +2503,7 @@
       <c r="X25" s="2" t="n"/>
       <c r="Y25" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -2582,7 +2582,7 @@
       <c r="X26" s="2" t="n"/>
       <c r="Y26" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -2661,7 +2661,7 @@
       <c r="X27" s="2" t="n"/>
       <c r="Y27" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -2740,7 +2740,7 @@
       <c r="X28" s="2" t="n"/>
       <c r="Y28" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -2819,7 +2819,7 @@
       <c r="X29" s="2" t="n"/>
       <c r="Y29" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -2898,7 +2898,7 @@
       <c r="X30" s="2" t="n"/>
       <c r="Y30" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -2977,7 +2977,7 @@
       <c r="X31" s="2" t="n"/>
       <c r="Y31" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -3056,7 +3056,7 @@
       <c r="X32" s="2" t="n"/>
       <c r="Y32" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -3135,7 +3135,7 @@
       <c r="X33" s="2" t="n"/>
       <c r="Y33" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -3214,7 +3214,7 @@
       <c r="X34" s="2" t="n"/>
       <c r="Y34" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -3293,7 +3293,7 @@
       <c r="X35" s="2" t="n"/>
       <c r="Y35" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -3372,7 +3372,7 @@
       <c r="X36" s="2" t="n"/>
       <c r="Y36" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -3451,7 +3451,7 @@
       <c r="X37" s="2" t="n"/>
       <c r="Y37" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -3530,7 +3530,7 @@
       <c r="X38" s="2" t="n"/>
       <c r="Y38" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -3609,7 +3609,7 @@
       <c r="X39" s="2" t="n"/>
       <c r="Y39" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -3688,7 +3688,7 @@
       <c r="X40" s="2" t="n"/>
       <c r="Y40" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -3767,7 +3767,7 @@
       <c r="X41" s="2" t="n"/>
       <c r="Y41" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -3846,7 +3846,7 @@
       <c r="X42" s="2" t="n"/>
       <c r="Y42" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -3925,7 +3925,7 @@
       <c r="X43" s="2" t="n"/>
       <c r="Y43" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -4004,7 +4004,7 @@
       <c r="X44" s="2" t="n"/>
       <c r="Y44" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       <c r="X45" s="2" t="n"/>
       <c r="Y45" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -4162,7 +4162,7 @@
       <c r="X46" s="2" t="n"/>
       <c r="Y46" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -4241,7 +4241,7 @@
       <c r="X47" s="2" t="n"/>
       <c r="Y47" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -4320,7 +4320,7 @@
       <c r="X48" s="2" t="n"/>
       <c r="Y48" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -4399,7 +4399,7 @@
       <c r="X49" s="2" t="n"/>
       <c r="Y49" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -4478,7 +4478,7 @@
       <c r="X50" s="2" t="n"/>
       <c r="Y50" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -4557,7 +4557,7 @@
       <c r="X51" s="2" t="n"/>
       <c r="Y51" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -4636,7 +4636,7 @@
       <c r="X52" s="2" t="n"/>
       <c r="Y52" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -4715,7 +4715,7 @@
       <c r="X53" s="2" t="n"/>
       <c r="Y53" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -4794,7 +4794,7 @@
       <c r="X54" s="2" t="n"/>
       <c r="Y54" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -4873,7 +4873,7 @@
       <c r="X55" s="2" t="n"/>
       <c r="Y55" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -4952,7 +4952,7 @@
       <c r="X56" s="2" t="n"/>
       <c r="Y56" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -5031,7 +5031,7 @@
       <c r="X57" s="2" t="n"/>
       <c r="Y57" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -5110,7 +5110,7 @@
       <c r="X58" s="2" t="n"/>
       <c r="Y58" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -5189,7 +5189,7 @@
       <c r="X59" s="2" t="n"/>
       <c r="Y59" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -5268,7 +5268,7 @@
       <c r="X60" s="2" t="n"/>
       <c r="Y60" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -5347,7 +5347,7 @@
       <c r="X61" s="2" t="n"/>
       <c r="Y61" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -5426,7 +5426,7 @@
       <c r="X62" s="2" t="n"/>
       <c r="Y62" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -5505,7 +5505,7 @@
       <c r="X63" s="2" t="n"/>
       <c r="Y63" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -5584,7 +5584,7 @@
       <c r="X64" s="2" t="n"/>
       <c r="Y64" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -5663,7 +5663,7 @@
       <c r="X65" s="2" t="n"/>
       <c r="Y65" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -5738,7 +5738,7 @@
       <c r="X66" s="2" t="n"/>
       <c r="Y66" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -5817,7 +5817,7 @@
       <c r="X67" s="2" t="n"/>
       <c r="Y67" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -5896,7 +5896,7 @@
       <c r="X68" s="2" t="n"/>
       <c r="Y68" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -5975,7 +5975,7 @@
       <c r="X69" s="2" t="n"/>
       <c r="Y69" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -6054,7 +6054,7 @@
       <c r="X70" s="2" t="n"/>
       <c r="Y70" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -6133,7 +6133,7 @@
       <c r="X71" s="2" t="n"/>
       <c r="Y71" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -6212,7 +6212,7 @@
       <c r="X72" s="2" t="n"/>
       <c r="Y72" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -6291,7 +6291,7 @@
       <c r="X73" s="2" t="n"/>
       <c r="Y73" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -6370,7 +6370,7 @@
       <c r="X74" s="2" t="n"/>
       <c r="Y74" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -6449,7 +6449,7 @@
       <c r="X75" s="2" t="n"/>
       <c r="Y75" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -6528,7 +6528,7 @@
       <c r="X76" s="2" t="n"/>
       <c r="Y76" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -6607,7 +6607,7 @@
       <c r="X77" s="2" t="n"/>
       <c r="Y77" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -6686,7 +6686,7 @@
       <c r="X78" s="2" t="n"/>
       <c r="Y78" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -6765,7 +6765,7 @@
       <c r="X79" s="2" t="n"/>
       <c r="Y79" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -6844,7 +6844,7 @@
       <c r="X80" s="2" t="n"/>
       <c r="Y80" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -6923,7 +6923,7 @@
       <c r="X81" s="2" t="n"/>
       <c r="Y81" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       <c r="X82" s="2" t="n"/>
       <c r="Y82" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -7081,7 +7081,7 @@
       <c r="X83" s="2" t="n"/>
       <c r="Y83" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>
@@ -7160,7 +7160,7 @@
       <c r="X84" s="2" t="n"/>
       <c r="Y84" s="2" t="inlineStr">
         <is>
-          <t>Hombre</t>
+          <t>HOMBRE</t>
         </is>
       </c>
     </row>

</xml_diff>